<commit_message>
Sprint 5: fixed fcf_cagr_5yr null-only column in cashflow_intelligence.xlsx by wiring in the existing cagr_from_series engine
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:M93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,20 +459,25 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>fcf_cagr_5yr_flag</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>fcf_conversion_pct</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>distress_flag</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>deleveraging_flag</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>capital_allocation_label</t>
         </is>
@@ -511,16 +516,21 @@
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="n">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
         <v>75.36132140399174</v>
       </c>
-      <c r="J2" t="b">
-        <v>0</v>
-      </c>
       <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="b">
         <v>1</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -559,16 +569,21 @@
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="n">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
         <v>19.17352477674663</v>
       </c>
-      <c r="J3" t="b">
-        <v>0</v>
-      </c>
       <c r="K3" t="b">
         <v>0</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -607,16 +622,21 @@
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="n">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>DECLINE_TO_LOSS</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
         <v>-74.31660367407929</v>
       </c>
-      <c r="J4" t="b">
-        <v>0</v>
-      </c>
       <c r="K4" t="b">
         <v>0</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -655,16 +675,21 @@
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="n">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
         <v>-182.3858977862804</v>
       </c>
-      <c r="J5" t="b">
-        <v>0</v>
-      </c>
       <c r="K5" t="b">
         <v>0</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -703,17 +728,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="n">
+      <c r="H6" t="n">
+        <v>37.78973446864202</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="n">
         <v>52.92193213163128</v>
       </c>
-      <c r="J6" t="b">
-        <v>0</v>
-      </c>
       <c r="K6" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" t="b">
         <v>1</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -751,17 +779,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="n">
+      <c r="H7" t="n">
+        <v>30.71118060790721</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="n">
         <v>96.83454026771999</v>
       </c>
-      <c r="J7" t="b">
-        <v>0</v>
-      </c>
       <c r="K7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" t="b">
         <v>1</v>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Liquidating Assets</t>
         </is>
@@ -800,16 +831,21 @@
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="n">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>DECLINE_TO_LOSS</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
         <v>-51.48437500000001</v>
       </c>
-      <c r="J8" t="b">
-        <v>0</v>
-      </c>
       <c r="K8" t="b">
         <v>0</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L8" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -848,17 +884,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="n">
+      <c r="H9" t="n">
+        <v>14.5722412524085</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="n">
         <v>15.99832915622389</v>
       </c>
-      <c r="J9" t="b">
-        <v>0</v>
-      </c>
       <c r="K9" t="b">
         <v>0</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -897,17 +936,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="n">
+      <c r="H10" t="n">
+        <v>18.03587045363451</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
         <v>46.88200395517469</v>
       </c>
-      <c r="J10" t="b">
-        <v>0</v>
-      </c>
       <c r="K10" t="b">
         <v>0</v>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -934,14 +976,19 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="b">
-        <v>0</v>
-      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="b">
         <v>0</v>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>Pre-Revenue</t>
         </is>
@@ -980,16 +1027,21 @@
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="n">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>DECLINE_TO_LOSS</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
         <v>-38.36280736894816</v>
       </c>
-      <c r="J12" t="b">
+      <c r="K12" t="b">
         <v>1</v>
       </c>
-      <c r="K12" t="b">
-        <v>0</v>
-      </c>
-      <c r="L12" t="inlineStr">
+      <c r="L12" t="b">
+        <v>0</v>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -1027,17 +1079,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="n">
+      <c r="H13" t="n">
+        <v>23.98235048893478</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="n">
         <v>73.99885909868796</v>
       </c>
-      <c r="J13" t="b">
-        <v>0</v>
-      </c>
       <c r="K13" t="b">
         <v>0</v>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L13" t="b">
+        <v>0</v>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -1076,16 +1131,21 @@
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="n">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
         <v>-194.7708261996772</v>
       </c>
-      <c r="J14" t="b">
+      <c r="K14" t="b">
         <v>1</v>
       </c>
-      <c r="K14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L14" t="inlineStr">
+      <c r="L14" t="b">
+        <v>0</v>
+      </c>
+      <c r="M14" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -1123,17 +1183,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
+      <c r="H15" t="n">
+        <v>25.86754704441738</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="n">
         <v>94.04609475032009</v>
       </c>
-      <c r="J15" t="b">
-        <v>0</v>
-      </c>
       <c r="K15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" t="b">
         <v>1</v>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -1172,16 +1235,21 @@
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="n">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
         <v>-496.4966768122243</v>
       </c>
-      <c r="J16" t="b">
+      <c r="K16" t="b">
         <v>1</v>
       </c>
-      <c r="K16" t="b">
-        <v>0</v>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="L16" t="b">
+        <v>0</v>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -1220,16 +1288,21 @@
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
         <v>-17.03283084341693</v>
       </c>
-      <c r="J17" t="b">
+      <c r="K17" t="b">
         <v>1</v>
       </c>
-      <c r="K17" t="b">
-        <v>0</v>
-      </c>
-      <c r="L17" t="inlineStr">
+      <c r="L17" t="b">
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -1268,16 +1341,21 @@
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>DECLINE_TO_LOSS</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
         <v>-25.04454563452781</v>
       </c>
-      <c r="J18" t="b">
-        <v>0</v>
-      </c>
       <c r="K18" t="b">
         <v>0</v>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L18" t="b">
+        <v>0</v>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -1316,16 +1394,21 @@
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
         <v>35.51959331732489</v>
       </c>
-      <c r="J19" t="b">
-        <v>0</v>
-      </c>
       <c r="K19" t="b">
+        <v>0</v>
+      </c>
+      <c r="L19" t="b">
         <v>1</v>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -1365,16 +1448,21 @@
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
         <v>-335.0210970464135</v>
       </c>
-      <c r="J20" t="b">
+      <c r="K20" t="b">
         <v>1</v>
       </c>
-      <c r="K20" t="b">
-        <v>0</v>
-      </c>
-      <c r="L20" t="inlineStr">
+      <c r="L20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>Distress Signal</t>
         </is>
@@ -1412,17 +1500,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="n">
+      <c r="H21" t="n">
+        <v>-8.223254104876499</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="n">
         <v>73.31742243436754</v>
       </c>
-      <c r="J21" t="b">
-        <v>0</v>
-      </c>
       <c r="K21" t="b">
+        <v>0</v>
+      </c>
+      <c r="L21" t="b">
         <v>1</v>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>Liquidating Assets</t>
         </is>
@@ -1461,16 +1552,21 @@
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="n">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
         <v>57.65391769883399</v>
       </c>
-      <c r="J22" t="b">
-        <v>0</v>
-      </c>
       <c r="K22" t="b">
+        <v>0</v>
+      </c>
+      <c r="L22" t="b">
         <v>1</v>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -1508,17 +1604,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="n">
+      <c r="H23" t="n">
+        <v>58.59345160881666</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="n">
         <v>96.30565203662772</v>
       </c>
-      <c r="J23" t="b">
-        <v>0</v>
-      </c>
       <c r="K23" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" t="b">
         <v>1</v>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>Liquidating Assets</t>
         </is>
@@ -1556,17 +1655,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="n">
+      <c r="H24" t="n">
+        <v>-5.337862323751841</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="n">
         <v>28.81289819269276</v>
       </c>
-      <c r="J24" t="b">
-        <v>0</v>
-      </c>
       <c r="K24" t="b">
         <v>0</v>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L24" t="b">
+        <v>0</v>
+      </c>
+      <c r="M24" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -1605,16 +1707,21 @@
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="n">
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
         <v>-715.6545961002786</v>
       </c>
-      <c r="J25" t="b">
+      <c r="K25" t="b">
         <v>1</v>
       </c>
-      <c r="K25" t="b">
-        <v>0</v>
-      </c>
-      <c r="L25" t="inlineStr">
+      <c r="L25" t="b">
+        <v>0</v>
+      </c>
+      <c r="M25" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -1653,17 +1760,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="n">
+      <c r="H26" t="n">
+        <v>228.7503659034452</v>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="n">
         <v>5.912847097469589</v>
       </c>
-      <c r="J26" t="b">
-        <v>0</v>
-      </c>
       <c r="K26" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" t="b">
         <v>1</v>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -1701,17 +1811,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="n">
+      <c r="H27" t="n">
+        <v>9.987217411819094</v>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="n">
         <v>14.43212650500254</v>
       </c>
-      <c r="J27" t="b">
-        <v>0</v>
-      </c>
       <c r="K27" t="b">
         <v>0</v>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L27" t="b">
+        <v>0</v>
+      </c>
+      <c r="M27" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -1749,17 +1862,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="n">
+      <c r="H28" t="n">
+        <v>-10.72050757546945</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="n">
         <v>43.41666666666666</v>
       </c>
-      <c r="J28" t="b">
-        <v>0</v>
-      </c>
       <c r="K28" t="b">
         <v>0</v>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L28" t="b">
+        <v>0</v>
+      </c>
+      <c r="M28" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -1797,17 +1913,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="n">
+      <c r="H29" t="n">
+        <v>29.82307104777742</v>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="n">
         <v>44.8868778280543</v>
       </c>
-      <c r="J29" t="b">
-        <v>0</v>
-      </c>
       <c r="K29" t="b">
         <v>0</v>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L29" t="b">
+        <v>0</v>
+      </c>
+      <c r="M29" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -1845,17 +1964,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="n">
+      <c r="H30" t="n">
+        <v>-13.16733127538306</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="n">
         <v>47.55178907721281</v>
       </c>
-      <c r="J30" t="b">
-        <v>0</v>
-      </c>
       <c r="K30" t="b">
         <v>0</v>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L30" t="b">
+        <v>0</v>
+      </c>
+      <c r="M30" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -1894,16 +2016,21 @@
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="n">
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
         <v>6.770579639551875</v>
       </c>
-      <c r="J31" t="b">
-        <v>0</v>
-      </c>
       <c r="K31" t="b">
         <v>0</v>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L31" t="b">
+        <v>0</v>
+      </c>
+      <c r="M31" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -1941,17 +2068,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="n">
+      <c r="H32" t="n">
+        <v>-24.68901184980715</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="n">
         <v>6.416235976301525</v>
       </c>
-      <c r="J32" t="b">
-        <v>0</v>
-      </c>
       <c r="K32" t="b">
         <v>0</v>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M32" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -1989,17 +2119,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="n">
+      <c r="H33" t="n">
+        <v>-0.552520013345259</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="n">
         <v>20.55902055902056</v>
       </c>
-      <c r="J33" t="b">
-        <v>0</v>
-      </c>
       <c r="K33" t="b">
         <v>0</v>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M33" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -2037,17 +2170,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="n">
+      <c r="H34" t="n">
+        <v>13.81411233198175</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="n">
         <v>30.45968981416794</v>
       </c>
-      <c r="J34" t="b">
-        <v>0</v>
-      </c>
       <c r="K34" t="b">
         <v>0</v>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L34" t="b">
+        <v>0</v>
+      </c>
+      <c r="M34" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2086,16 +2222,21 @@
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="n">
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>DECLINE_TO_LOSS</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
         <v>-46.16165032127156</v>
       </c>
-      <c r="J35" t="b">
-        <v>0</v>
-      </c>
       <c r="K35" t="b">
         <v>0</v>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M35" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -2134,16 +2275,21 @@
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="n">
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
         <v>-124.408898694613</v>
       </c>
-      <c r="J36" t="b">
+      <c r="K36" t="b">
         <v>1</v>
       </c>
-      <c r="K36" t="b">
-        <v>0</v>
-      </c>
-      <c r="L36" t="inlineStr">
+      <c r="L36" t="b">
+        <v>0</v>
+      </c>
+      <c r="M36" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -2182,16 +2328,21 @@
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="n">
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
         <v>18.60703661914042</v>
       </c>
-      <c r="J37" t="b">
-        <v>0</v>
-      </c>
       <c r="K37" t="b">
         <v>0</v>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L37" t="b">
+        <v>0</v>
+      </c>
+      <c r="M37" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2229,17 +2380,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="n">
+      <c r="H38" t="n">
+        <v>-13.35487386941974</v>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="n">
         <v>17.80967570441255</v>
       </c>
-      <c r="J38" t="b">
-        <v>0</v>
-      </c>
       <c r="K38" t="b">
         <v>0</v>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L38" t="b">
+        <v>0</v>
+      </c>
+      <c r="M38" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2277,17 +2431,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="n">
+      <c r="H39" t="n">
+        <v>22.6161818543015</v>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="n">
         <v>65.45995536821225</v>
       </c>
-      <c r="J39" t="b">
-        <v>0</v>
-      </c>
       <c r="K39" t="b">
         <v>0</v>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L39" t="b">
+        <v>0</v>
+      </c>
+      <c r="M39" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2326,16 +2483,21 @@
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="n">
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
         <v>20.47635996234127</v>
       </c>
-      <c r="J40" t="b">
-        <v>0</v>
-      </c>
       <c r="K40" t="b">
         <v>0</v>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="L40" t="b">
+        <v>0</v>
+      </c>
+      <c r="M40" t="inlineStr">
         <is>
           <t>Liquidating Assets</t>
         </is>
@@ -2374,16 +2536,21 @@
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="n">
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
         <v>-2.865746748422502</v>
       </c>
-      <c r="J41" t="b">
-        <v>0</v>
-      </c>
       <c r="K41" t="b">
         <v>0</v>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L41" t="b">
+        <v>0</v>
+      </c>
+      <c r="M41" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2422,17 +2589,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="n">
+      <c r="H42" t="n">
+        <v>5.842708892319703</v>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="n">
         <v>9.507280211341156</v>
       </c>
-      <c r="J42" t="b">
-        <v>0</v>
-      </c>
       <c r="K42" t="b">
         <v>0</v>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L42" t="b">
+        <v>0</v>
+      </c>
+      <c r="M42" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2470,17 +2640,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="n">
+      <c r="H43" t="n">
+        <v>8.463802473474736</v>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="n">
         <v>5.096048727159144</v>
       </c>
-      <c r="J43" t="b">
-        <v>0</v>
-      </c>
       <c r="K43" t="b">
         <v>0</v>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L43" t="b">
+        <v>0</v>
+      </c>
+      <c r="M43" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2519,17 +2692,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="n">
+      <c r="H44" t="n">
+        <v>13.60175699592767</v>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="n">
         <v>21.47680843406652</v>
       </c>
-      <c r="J44" t="b">
-        <v>0</v>
-      </c>
       <c r="K44" t="b">
         <v>0</v>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L44" t="b">
+        <v>0</v>
+      </c>
+      <c r="M44" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2567,17 +2743,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="n">
+      <c r="H45" t="n">
+        <v>-7.360467011220518</v>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="n">
         <v>12.60245078344717</v>
       </c>
-      <c r="J45" t="b">
-        <v>0</v>
-      </c>
       <c r="K45" t="b">
         <v>0</v>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L45" t="b">
+        <v>0</v>
+      </c>
+      <c r="M45" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -2615,17 +2794,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="n">
+      <c r="H46" t="n">
+        <v>32.27903093325808</v>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="n">
         <v>2.71356783919598</v>
       </c>
-      <c r="J46" t="b">
-        <v>0</v>
-      </c>
       <c r="K46" t="b">
+        <v>0</v>
+      </c>
+      <c r="L46" t="b">
         <v>1</v>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2663,17 +2845,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="n">
+      <c r="H47" t="n">
+        <v>-51.26166654001434</v>
+      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="n">
         <v>0.1139619692628289</v>
       </c>
-      <c r="J47" t="b">
-        <v>0</v>
-      </c>
       <c r="K47" t="b">
+        <v>0</v>
+      </c>
+      <c r="L47" t="b">
         <v>1</v>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="M47" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -2711,17 +2896,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="n">
+      <c r="H48" t="n">
+        <v>71.56520119992503</v>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="n">
         <v>17.92555113841706</v>
       </c>
-      <c r="J48" t="b">
-        <v>0</v>
-      </c>
       <c r="K48" t="b">
         <v>0</v>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L48" t="b">
+        <v>0</v>
+      </c>
+      <c r="M48" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2760,16 +2948,21 @@
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="n">
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
         <v>-99.03617190157614</v>
       </c>
-      <c r="J49" t="b">
-        <v>0</v>
-      </c>
       <c r="K49" t="b">
         <v>0</v>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L49" t="b">
+        <v>0</v>
+      </c>
+      <c r="M49" t="inlineStr">
         <is>
           <t>Pre-Revenue</t>
         </is>
@@ -2807,17 +3000,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="n">
+      <c r="H50" t="n">
+        <v>7.201272446841034</v>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="n">
         <v>55.22855181880576</v>
       </c>
-      <c r="J50" t="b">
-        <v>0</v>
-      </c>
       <c r="K50" t="b">
         <v>0</v>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="L50" t="b">
+        <v>0</v>
+      </c>
+      <c r="M50" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -2857,16 +3053,21 @@
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="n">
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
         <v>52.39536789783994</v>
       </c>
-      <c r="J51" t="b">
-        <v>0</v>
-      </c>
       <c r="K51" t="b">
         <v>0</v>
       </c>
-      <c r="L51" t="inlineStr">
+      <c r="L51" t="b">
+        <v>0</v>
+      </c>
+      <c r="M51" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -2904,17 +3105,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="n">
+      <c r="H52" t="n">
+        <v>35.50477381816852</v>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="n">
         <v>45.49795361527968</v>
       </c>
-      <c r="J52" t="b">
-        <v>0</v>
-      </c>
       <c r="K52" t="b">
+        <v>0</v>
+      </c>
+      <c r="L52" t="b">
         <v>1</v>
       </c>
-      <c r="L52" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -2953,16 +3157,21 @@
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="n">
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
         <v>29.81933391166598</v>
       </c>
-      <c r="J53" t="b">
-        <v>0</v>
-      </c>
       <c r="K53" t="b">
+        <v>0</v>
+      </c>
+      <c r="L53" t="b">
         <v>1</v>
       </c>
-      <c r="L53" t="inlineStr">
+      <c r="M53" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -3001,17 +3210,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="n">
+      <c r="H54" t="n">
+        <v>21.64259503734181</v>
+      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="n">
         <v>71.44436396904662</v>
       </c>
-      <c r="J54" t="b">
-        <v>0</v>
-      </c>
       <c r="K54" t="b">
+        <v>0</v>
+      </c>
+      <c r="L54" t="b">
         <v>1</v>
       </c>
-      <c r="L54" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>Liquidating Assets</t>
         </is>
@@ -3050,16 +3262,21 @@
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="n">
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>DECLINE_TO_LOSS</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
         <v>-22.89747108410116</v>
       </c>
-      <c r="J55" t="b">
-        <v>0</v>
-      </c>
       <c r="K55" t="b">
         <v>0</v>
       </c>
-      <c r="L55" t="inlineStr">
+      <c r="L55" t="b">
+        <v>0</v>
+      </c>
+      <c r="M55" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -3098,16 +3315,21 @@
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
-      <c r="I56" t="n">
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
         <v>48.94162924951892</v>
       </c>
-      <c r="J56" t="b">
-        <v>0</v>
-      </c>
       <c r="K56" t="b">
+        <v>0</v>
+      </c>
+      <c r="L56" t="b">
         <v>1</v>
       </c>
-      <c r="L56" t="inlineStr">
+      <c r="M56" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -3146,16 +3368,21 @@
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
-      <c r="I57" t="n">
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>DECLINE_TO_LOSS</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
         <v>-36.47342995169083</v>
       </c>
-      <c r="J57" t="b">
-        <v>0</v>
-      </c>
       <c r="K57" t="b">
         <v>0</v>
       </c>
-      <c r="L57" t="inlineStr">
+      <c r="L57" t="b">
+        <v>0</v>
+      </c>
+      <c r="M57" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -3194,16 +3421,21 @@
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
-      <c r="I58" t="n">
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>DECLINE_TO_LOSS</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
         <v>-8.484568668537131</v>
       </c>
-      <c r="J58" t="b">
-        <v>0</v>
-      </c>
       <c r="K58" t="b">
         <v>0</v>
       </c>
-      <c r="L58" t="inlineStr">
+      <c r="L58" t="b">
+        <v>0</v>
+      </c>
+      <c r="M58" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -3243,16 +3475,21 @@
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
-      <c r="I59" t="n">
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
         <v>14.37983507608603</v>
       </c>
-      <c r="J59" t="b">
-        <v>0</v>
-      </c>
       <c r="K59" t="b">
         <v>0</v>
       </c>
-      <c r="L59" t="inlineStr">
+      <c r="L59" t="b">
+        <v>0</v>
+      </c>
+      <c r="M59" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -3290,17 +3527,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="n">
+      <c r="H60" t="n">
+        <v>-48.21728841371581</v>
+      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="n">
         <v>2.602275847341285</v>
       </c>
-      <c r="J60" t="b">
-        <v>0</v>
-      </c>
       <c r="K60" t="b">
         <v>0</v>
       </c>
-      <c r="L60" t="inlineStr">
+      <c r="L60" t="b">
+        <v>0</v>
+      </c>
+      <c r="M60" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -3339,16 +3579,21 @@
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
-      <c r="I61" t="n">
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
         <v>-16.32270168855535</v>
       </c>
-      <c r="J61" t="b">
-        <v>0</v>
-      </c>
       <c r="K61" t="b">
         <v>0</v>
       </c>
-      <c r="L61" t="inlineStr">
+      <c r="L61" t="b">
+        <v>0</v>
+      </c>
+      <c r="M61" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -3387,16 +3632,21 @@
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="n">
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
         <v>68.45806127574083</v>
       </c>
-      <c r="J62" t="b">
-        <v>0</v>
-      </c>
       <c r="K62" t="b">
         <v>0</v>
       </c>
-      <c r="L62" t="inlineStr">
+      <c r="L62" t="b">
+        <v>0</v>
+      </c>
+      <c r="M62" t="inlineStr">
         <is>
           <t>Liquidating Assets</t>
         </is>
@@ -3434,17 +3684,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="n">
+      <c r="H63" t="n">
+        <v>22.08444037386408</v>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="n">
         <v>27.43071864725223</v>
       </c>
-      <c r="J63" t="b">
-        <v>0</v>
-      </c>
       <c r="K63" t="b">
         <v>0</v>
       </c>
-      <c r="L63" t="inlineStr">
+      <c r="L63" t="b">
+        <v>0</v>
+      </c>
+      <c r="M63" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -3484,16 +3737,21 @@
         </is>
       </c>
       <c r="H64" t="inlineStr"/>
-      <c r="I64" t="n">
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
         <v>-45.17515667684396</v>
       </c>
-      <c r="J64" t="b">
+      <c r="K64" t="b">
         <v>1</v>
       </c>
-      <c r="K64" t="b">
-        <v>0</v>
-      </c>
-      <c r="L64" t="inlineStr">
+      <c r="L64" t="b">
+        <v>0</v>
+      </c>
+      <c r="M64" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -3531,17 +3789,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="n">
+      <c r="H65" t="n">
+        <v>10.02778351575371</v>
+      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="n">
         <v>26.50059057231827</v>
       </c>
-      <c r="J65" t="b">
-        <v>0</v>
-      </c>
       <c r="K65" t="b">
+        <v>0</v>
+      </c>
+      <c r="L65" t="b">
         <v>1</v>
       </c>
-      <c r="L65" t="inlineStr">
+      <c r="M65" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -3579,17 +3840,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="n">
+      <c r="H66" t="n">
+        <v>-1.428567128563307</v>
+      </c>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="n">
         <v>9.922763355503111</v>
       </c>
-      <c r="J66" t="b">
-        <v>0</v>
-      </c>
       <c r="K66" t="b">
         <v>0</v>
       </c>
-      <c r="L66" t="inlineStr">
+      <c r="L66" t="b">
+        <v>0</v>
+      </c>
+      <c r="M66" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -3628,16 +3892,21 @@
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
-      <c r="I67" t="n">
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>DECLINE_TO_LOSS</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
         <v>-21.09704641350211</v>
       </c>
-      <c r="J67" t="b">
-        <v>0</v>
-      </c>
       <c r="K67" t="b">
         <v>0</v>
       </c>
-      <c r="L67" t="inlineStr">
+      <c r="L67" t="b">
+        <v>0</v>
+      </c>
+      <c r="M67" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -3675,17 +3944,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="n">
+      <c r="H68" t="n">
+        <v>4.320098447494725</v>
+      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="n">
         <v>50.54188886977465</v>
       </c>
-      <c r="J68" t="b">
-        <v>0</v>
-      </c>
       <c r="K68" t="b">
         <v>0</v>
       </c>
-      <c r="L68" t="inlineStr">
+      <c r="L68" t="b">
+        <v>0</v>
+      </c>
+      <c r="M68" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -3724,17 +3996,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="n">
+      <c r="H69" t="n">
+        <v>-18.15959230256928</v>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="n">
         <v>20.17890576242979</v>
       </c>
-      <c r="J69" t="b">
-        <v>0</v>
-      </c>
       <c r="K69" t="b">
         <v>0</v>
       </c>
-      <c r="L69" t="inlineStr">
+      <c r="L69" t="b">
+        <v>0</v>
+      </c>
+      <c r="M69" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -3773,16 +4048,21 @@
         </is>
       </c>
       <c r="H70" t="inlineStr"/>
-      <c r="I70" t="n">
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
         <v>16.7988184079602</v>
       </c>
-      <c r="J70" t="b">
-        <v>0</v>
-      </c>
       <c r="K70" t="b">
         <v>0</v>
       </c>
-      <c r="L70" t="inlineStr">
+      <c r="L70" t="b">
+        <v>0</v>
+      </c>
+      <c r="M70" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -3820,17 +4100,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="n">
+      <c r="H71" t="n">
+        <v>11.57315479777334</v>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="n">
         <v>40.90047162930909</v>
       </c>
-      <c r="J71" t="b">
-        <v>0</v>
-      </c>
       <c r="K71" t="b">
         <v>0</v>
       </c>
-      <c r="L71" t="inlineStr">
+      <c r="L71" t="b">
+        <v>0</v>
+      </c>
+      <c r="M71" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -3869,16 +4152,21 @@
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
-      <c r="I72" t="n">
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
         <v>-301.5190778303994</v>
       </c>
-      <c r="J72" t="b">
+      <c r="K72" t="b">
         <v>1</v>
       </c>
-      <c r="K72" t="b">
-        <v>0</v>
-      </c>
-      <c r="L72" t="inlineStr">
+      <c r="L72" t="b">
+        <v>0</v>
+      </c>
+      <c r="M72" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -3916,17 +4204,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="n">
+      <c r="H73" t="n">
+        <v>23.53017525858574</v>
+      </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="n">
         <v>35.2658788774003</v>
       </c>
-      <c r="J73" t="b">
-        <v>0</v>
-      </c>
       <c r="K73" t="b">
+        <v>0</v>
+      </c>
+      <c r="L73" t="b">
         <v>1</v>
       </c>
-      <c r="L73" t="inlineStr">
+      <c r="M73" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -3965,14 +4256,19 @@
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="b">
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="b">
         <v>1</v>
       </c>
-      <c r="K74" t="b">
-        <v>0</v>
-      </c>
-      <c r="L74" t="inlineStr">
+      <c r="L74" t="b">
+        <v>0</v>
+      </c>
+      <c r="M74" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -4010,17 +4306,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="n">
+      <c r="H75" t="n">
+        <v>39.69769001638159</v>
+      </c>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="n">
         <v>60.70406267262592</v>
       </c>
-      <c r="J75" t="b">
-        <v>0</v>
-      </c>
       <c r="K75" t="b">
+        <v>0</v>
+      </c>
+      <c r="L75" t="b">
         <v>1</v>
       </c>
-      <c r="L75" t="inlineStr">
+      <c r="M75" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -4059,16 +4358,21 @@
         </is>
       </c>
       <c r="H76" t="inlineStr"/>
-      <c r="I76" t="n">
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
         <v>-124.3739949460142</v>
       </c>
-      <c r="J76" t="b">
+      <c r="K76" t="b">
         <v>1</v>
       </c>
-      <c r="K76" t="b">
-        <v>0</v>
-      </c>
-      <c r="L76" t="inlineStr">
+      <c r="L76" t="b">
+        <v>0</v>
+      </c>
+      <c r="M76" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -4108,16 +4412,21 @@
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
-      <c r="I77" t="n">
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
         <v>27.82003470811948</v>
       </c>
-      <c r="J77" t="b">
-        <v>0</v>
-      </c>
       <c r="K77" t="b">
+        <v>0</v>
+      </c>
+      <c r="L77" t="b">
         <v>1</v>
       </c>
-      <c r="L77" t="inlineStr">
+      <c r="M77" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -4156,16 +4465,21 @@
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
-      <c r="I78" t="n">
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
         <v>-853.2520325203253</v>
       </c>
-      <c r="J78" t="b">
-        <v>0</v>
-      </c>
       <c r="K78" t="b">
         <v>0</v>
       </c>
-      <c r="L78" t="inlineStr">
+      <c r="L78" t="b">
+        <v>0</v>
+      </c>
+      <c r="M78" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -4203,17 +4517,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="n">
+      <c r="H79" t="n">
+        <v>-9.42032384113779</v>
+      </c>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="n">
         <v>-30.11095079357182</v>
       </c>
-      <c r="J79" t="b">
-        <v>0</v>
-      </c>
       <c r="K79" t="b">
         <v>0</v>
       </c>
-      <c r="L79" t="inlineStr">
+      <c r="L79" t="b">
+        <v>0</v>
+      </c>
+      <c r="M79" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -4251,17 +4568,20 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="n">
+      <c r="H80" t="n">
+        <v>7.24045892978542</v>
+      </c>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="n">
         <v>42.69588313413015</v>
       </c>
-      <c r="J80" t="b">
-        <v>0</v>
-      </c>
       <c r="K80" t="b">
+        <v>0</v>
+      </c>
+      <c r="L80" t="b">
         <v>1</v>
       </c>
-      <c r="L80" t="inlineStr">
+      <c r="M80" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -4301,16 +4621,21 @@
         </is>
       </c>
       <c r="H81" t="inlineStr"/>
-      <c r="I81" t="n">
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
         <v>-298.0043713769838</v>
       </c>
-      <c r="J81" t="b">
+      <c r="K81" t="b">
         <v>1</v>
       </c>
-      <c r="K81" t="b">
-        <v>0</v>
-      </c>
-      <c r="L81" t="inlineStr">
+      <c r="L81" t="b">
+        <v>0</v>
+      </c>
+      <c r="M81" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>
@@ -4348,17 +4673,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="n">
+      <c r="H82" t="n">
+        <v>53.28962129081927</v>
+      </c>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="n">
         <v>37.62886597938144</v>
       </c>
-      <c r="J82" t="b">
-        <v>0</v>
-      </c>
       <c r="K82" t="b">
         <v>0</v>
       </c>
-      <c r="L82" t="inlineStr">
+      <c r="L82" t="b">
+        <v>0</v>
+      </c>
+      <c r="M82" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -4396,17 +4724,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="n">
+      <c r="H83" t="n">
+        <v>43.2382586094409</v>
+      </c>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="n">
         <v>87.35596865878014</v>
       </c>
-      <c r="J83" t="b">
-        <v>0</v>
-      </c>
       <c r="K83" t="b">
+        <v>0</v>
+      </c>
+      <c r="L83" t="b">
         <v>1</v>
       </c>
-      <c r="L83" t="inlineStr">
+      <c r="M83" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -4444,17 +4775,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="n">
+      <c r="H84" t="n">
+        <v>-37.04887150623013</v>
+      </c>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="n">
         <v>1.138353765323993</v>
       </c>
-      <c r="J84" t="b">
-        <v>0</v>
-      </c>
       <c r="K84" t="b">
         <v>0</v>
       </c>
-      <c r="L84" t="inlineStr">
+      <c r="L84" t="b">
+        <v>0</v>
+      </c>
+      <c r="M84" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -4493,16 +4827,21 @@
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
-      <c r="I85" t="n">
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
         <v>75.80536800026874</v>
       </c>
-      <c r="J85" t="b">
-        <v>0</v>
-      </c>
       <c r="K85" t="b">
+        <v>0</v>
+      </c>
+      <c r="L85" t="b">
         <v>1</v>
       </c>
-      <c r="L85" t="inlineStr">
+      <c r="M85" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -4541,17 +4880,20 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="n">
+      <c r="H86" t="n">
+        <v>-3.666968259247616</v>
+      </c>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="n">
         <v>33.24639031206335</v>
       </c>
-      <c r="J86" t="b">
-        <v>0</v>
-      </c>
       <c r="K86" t="b">
         <v>0</v>
       </c>
-      <c r="L86" t="inlineStr">
+      <c r="L86" t="b">
+        <v>0</v>
+      </c>
+      <c r="M86" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -4591,16 +4933,21 @@
         </is>
       </c>
       <c r="H87" t="inlineStr"/>
-      <c r="I87" t="n">
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
         <v>27.18446601941747</v>
       </c>
-      <c r="J87" t="b">
-        <v>0</v>
-      </c>
       <c r="K87" t="b">
         <v>0</v>
       </c>
-      <c r="L87" t="inlineStr">
+      <c r="L87" t="b">
+        <v>0</v>
+      </c>
+      <c r="M87" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -4638,17 +4985,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="n">
+      <c r="H88" t="n">
+        <v>10.77084245698778</v>
+      </c>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="n">
         <v>78.43256190120692</v>
       </c>
-      <c r="J88" t="b">
-        <v>0</v>
-      </c>
       <c r="K88" t="b">
         <v>0</v>
       </c>
-      <c r="L88" t="inlineStr">
+      <c r="L88" t="b">
+        <v>0</v>
+      </c>
+      <c r="M88" t="inlineStr">
         <is>
           <t>Liquidating Assets</t>
         </is>
@@ -4686,17 +5036,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="n">
+      <c r="H89" t="n">
+        <v>16.78825509724664</v>
+      </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="n">
         <v>112.2503328894807</v>
       </c>
-      <c r="J89" t="b">
-        <v>0</v>
-      </c>
       <c r="K89" t="b">
+        <v>0</v>
+      </c>
+      <c r="L89" t="b">
         <v>1</v>
       </c>
-      <c r="L89" t="inlineStr">
+      <c r="M89" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -4735,17 +5088,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="n">
+      <c r="H90" t="n">
+        <v>27.55515729109304</v>
+      </c>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="n">
         <v>28.45804988662132</v>
       </c>
-      <c r="J90" t="b">
-        <v>0</v>
-      </c>
       <c r="K90" t="b">
         <v>0</v>
       </c>
-      <c r="L90" t="inlineStr">
+      <c r="L90" t="b">
+        <v>0</v>
+      </c>
+      <c r="M90" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -4783,17 +5139,20 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="n">
+      <c r="H91" t="n">
+        <v>14.88463449987261</v>
+      </c>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="n">
         <v>92.22090261282661</v>
       </c>
-      <c r="J91" t="b">
-        <v>0</v>
-      </c>
       <c r="K91" t="b">
+        <v>0</v>
+      </c>
+      <c r="L91" t="b">
         <v>1</v>
       </c>
-      <c r="L91" t="inlineStr">
+      <c r="M91" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
@@ -4832,16 +5191,21 @@
         </is>
       </c>
       <c r="H92" t="inlineStr"/>
-      <c r="I92" t="n">
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>TURNAROUND</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
         <v>42.66869609335362</v>
       </c>
-      <c r="J92" t="b">
-        <v>0</v>
-      </c>
       <c r="K92" t="b">
+        <v>0</v>
+      </c>
+      <c r="L92" t="b">
         <v>1</v>
       </c>
-      <c r="L92" t="inlineStr">
+      <c r="M92" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -4880,16 +5244,21 @@
         </is>
       </c>
       <c r="H93" t="inlineStr"/>
-      <c r="I93" t="n">
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>BOTH_NEGATIVE</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
         <v>-40.98181818181818</v>
       </c>
-      <c r="J93" t="b">
+      <c r="K93" t="b">
         <v>1</v>
       </c>
-      <c r="K93" t="b">
-        <v>0</v>
-      </c>
-      <c r="L93" t="inlineStr">
+      <c r="L93" t="b">
+        <v>0</v>
+      </c>
+      <c r="M93" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>

</xml_diff>